<commit_message>
Update workbook and HTML structure for improved data accuracy and accessibility
- Replaced the existing `workbook.xlsx` file to ensure data consistency across the documentation.
- Updated table IDs and styling in the demographics, mortality, and SDOH chapters for better navigation and user experience.

These changes enhance the integrity of the data and improve the overall usability of the Community Health Assessment documentation.
</commit_message>
<xml_diff>
--- a/data/raw/workbook.xlsx
+++ b/data/raw/workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Work Drive/GitHub/Orange County CHA/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42E6EF7-BB5D-874E-89F4-E4888F087A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FA1F964-AC33-2B48-A596-B42D701C24AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" firstSheet="23" activeTab="31" xr2:uid="{7B5489DC-BB92-4237-A1A8-C16ED0406E77}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" firstSheet="17" activeTab="20" xr2:uid="{7B5489DC-BB92-4237-A1A8-C16ED0406E77}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -5682,11 +5682,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -18126,26 +18126,26 @@
       <c r="G10" s="24">
         <v>113465</v>
       </c>
-      <c r="H10" s="60">
+      <c r="H10" s="59">
         <v>26215</v>
       </c>
-      <c r="I10" s="60"/>
-      <c r="J10" s="60">
+      <c r="I10" s="59"/>
+      <c r="J10" s="59">
         <v>21762</v>
       </c>
-      <c r="K10" s="60"/>
-      <c r="L10" s="60">
+      <c r="K10" s="59"/>
+      <c r="L10" s="59">
         <v>6666</v>
       </c>
-      <c r="M10" s="60"/>
-      <c r="N10" s="60">
+      <c r="M10" s="59"/>
+      <c r="N10" s="59">
         <v>6666</v>
       </c>
-      <c r="O10" s="60"/>
-      <c r="P10" s="60">
+      <c r="O10" s="59"/>
+      <c r="P10" s="59">
         <v>4602</v>
       </c>
-      <c r="Q10" s="60"/>
+      <c r="Q10" s="59"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -18204,7 +18204,7 @@
         <v>1312</v>
       </c>
       <c r="O12" s="54"/>
-      <c r="P12" s="59" t="s">
+      <c r="P12" s="60" t="s">
         <v>1322</v>
       </c>
       <c r="Q12" s="54"/>
@@ -18220,26 +18220,26 @@
       <c r="G13" s="15">
         <v>173986</v>
       </c>
-      <c r="H13" s="60">
+      <c r="H13" s="59">
         <v>43166</v>
       </c>
-      <c r="I13" s="60"/>
-      <c r="J13" s="60">
+      <c r="I13" s="59"/>
+      <c r="J13" s="59">
         <v>32584</v>
       </c>
-      <c r="K13" s="60"/>
-      <c r="L13" s="60">
+      <c r="K13" s="59"/>
+      <c r="L13" s="59">
         <v>11174</v>
       </c>
-      <c r="M13" s="60"/>
-      <c r="N13" s="60">
+      <c r="M13" s="59"/>
+      <c r="N13" s="59">
         <v>10820</v>
       </c>
-      <c r="O13" s="60"/>
-      <c r="P13" s="60">
+      <c r="O13" s="59"/>
+      <c r="P13" s="59">
         <v>6574</v>
       </c>
-      <c r="Q13" s="60"/>
+      <c r="Q13" s="59"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -18490,51 +18490,6 @@
     </row>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="P14:Q14"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="P10:Q10"/>
-    <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="P9:Q9"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="P5:Q5"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="N6:O6"/>
-    <mergeCell ref="P6:Q6"/>
     <mergeCell ref="B1:O1"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="E5:E57"/>
@@ -18551,6 +18506,51 @@
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="N7:O7"/>
     <mergeCell ref="N8:O8"/>
+    <mergeCell ref="P5:Q5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="P14:Q14"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="P11:Q11"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10" xr:uid="{F82E15B8-D06A-4152-8A77-8AE50325986B}">
@@ -25072,6 +25072,9 @@
       <c r="A11" t="s">
         <v>262</v>
       </c>
+      <c r="B11" t="s">
+        <v>1305</v>
+      </c>
       <c r="E11" s="52"/>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
@@ -25087,7 +25090,7 @@
         <v>263</v>
       </c>
       <c r="B12" t="s">
-        <v>1305</v>
+        <v>1302</v>
       </c>
       <c r="E12" s="52"/>
       <c r="F12" s="22"/>
@@ -25101,9 +25104,6 @@
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>264</v>
-      </c>
-      <c r="B13" t="s">
-        <v>1302</v>
       </c>
       <c r="E13" s="52"/>
     </row>
@@ -32567,6 +32567,14 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B1:O1"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="E5:E57"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="H5:N5"/>
     <mergeCell ref="P6:Q6"/>
     <mergeCell ref="R6:S6"/>
     <mergeCell ref="T6:U6"/>
@@ -32576,14 +32584,6 @@
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="L6:M6"/>
     <mergeCell ref="N6:O6"/>
-    <mergeCell ref="B1:O1"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="E5:E57"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="H5:N5"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P4:U4" xr:uid="{0EF314E6-73BE-48BA-8EA7-0A11DA3A5308}">
@@ -74520,15 +74520,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="70db5d92-cf7a-41c9-a808-9efa4eb812f2">
@@ -74539,7 +74530,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005E06BBCF48891B4AA000B842D02367CE" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fe6ea1b7fa6cedb1acda08ea4d5bc607">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="70db5d92-cf7a-41c9-a808-9efa4eb812f2" xmlns:ns3="be71ce3a-ef61-410b-aae3-59cf01e8169d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6c75d4e196960d1be8fe94f46d8363ec" ns2:_="" ns3:_="">
     <xsd:import namespace="70db5d92-cf7a-41c9-a808-9efa4eb812f2"/>
@@ -74740,15 +74731,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B32976BB-D998-4BA5-BBBA-603A232D7A40}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5179601-D499-4F72-B04B-030712A0A5FF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -74765,7 +74757,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F22F824-927F-48AC-8EEE-0CBA7B354FB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -74782,4 +74774,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B32976BB-D998-4BA5-BBBA-603A232D7A40}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>